<commit_message>
Update lrm namespace and properties dictionary
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/properties.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/properties.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10517"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dponti/GitHub/def/Codelist Excel Files and Conversion Templates to XML/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dponti/Documents/GitHub/def/Codelist Excel Files and Conversion Templates to XML/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21CA86EC-9D19-7C44-9B78-E990FE33F77A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B2F44E-23C8-2141-9CB5-BDB76AF1154E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20700" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10020" yWindow="2560" windowWidth="35840" windowHeight="20700" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DictionaryName" sheetId="3" r:id="rId1"/>
@@ -3065,7 +3065,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -3161,16 +3161,6 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -3270,6 +3260,38 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -3325,38 +3347,6 @@
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium7"/>
   <extLst>
@@ -3384,38 +3374,38 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DictionaryName" displayName="DictionaryName" ref="A1:E3" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DictionaryName" displayName="DictionaryName" ref="A1:E3" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:E3" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Start" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Dictionary ID" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Start" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Dictionary ID" dataDxfId="7"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="DictionaryFile"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DictionaryName" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DictionaryName" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Definitions" displayName="Definitions" ref="A1:J199" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Definitions" displayName="Definitions" ref="A1:J199" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="A1:J199" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H180">
     <sortCondition ref="B1:B180"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Start" dataDxfId="14">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Start" dataDxfId="20">
       <calculatedColumnFormula>IF(ISNA(VLOOKUP(B2,AssociatedElements!B$2:B659,1,FALSE)),"Not used","")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ID" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Name" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Description" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="DataType" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="QuantityClass" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Authority" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Reference" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{514A6BB8-33C8-4E31-A303-203B88580677}" name="SLD Comment" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{941837FD-9A64-45F5-AA1B-805F9901FDC7}" name="SLD Changed" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ID" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Name" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Description" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="DataType" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="QuantityClass" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Authority" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Reference" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{514A6BB8-33C8-4E31-A303-203B88580677}" name="SLD Comment" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{941837FD-9A64-45F5-AA1B-805F9901FDC7}" name="SLD Changed" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7784,7 +7774,7 @@
       </c>
     </row>
     <row r="190" spans="1:10" ht="34">
-      <c r="A190" s="39" t="str">
+      <c r="A190" s="2" t="str">
         <f>IF(ISNA(VLOOKUP(B190,AssociatedElements!B$2:B847,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
@@ -7794,18 +7784,18 @@
       <c r="C190" s="2" t="s">
         <v>892</v>
       </c>
-      <c r="D190" s="40" t="s">
+      <c r="D190" s="2" t="s">
         <v>893</v>
       </c>
       <c r="E190" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F190" s="41" t="s">
+      <c r="F190" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="191" spans="1:10" ht="34">
-      <c r="A191" s="39" t="str">
+      <c r="A191" s="2" t="str">
         <f>IF(ISNA(VLOOKUP(B191,AssociatedElements!B$2:B848,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
@@ -7815,18 +7805,18 @@
       <c r="C191" s="2" t="s">
         <v>894</v>
       </c>
-      <c r="D191" s="40" t="s">
+      <c r="D191" s="2" t="s">
         <v>895</v>
       </c>
       <c r="E191" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F191" s="41" t="s">
+      <c r="F191" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="192" spans="1:10" ht="34">
-      <c r="A192" s="39" t="str">
+      <c r="A192" s="2" t="str">
         <f>IF(ISNA(VLOOKUP(B192,AssociatedElements!B$2:B849,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
@@ -7836,18 +7826,18 @@
       <c r="C192" s="2" t="s">
         <v>897</v>
       </c>
-      <c r="D192" s="40" t="s">
+      <c r="D192" s="2" t="s">
         <v>898</v>
       </c>
       <c r="E192" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F192" s="41" t="s">
+      <c r="F192" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="193" spans="1:6" ht="34">
-      <c r="A193" s="39" t="str">
+      <c r="A193" s="2" t="str">
         <f>IF(ISNA(VLOOKUP(B193,AssociatedElements!B$2:B850,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
@@ -7857,18 +7847,18 @@
       <c r="C193" s="2" t="s">
         <v>900</v>
       </c>
-      <c r="D193" s="40" t="s">
+      <c r="D193" s="2" t="s">
         <v>901</v>
       </c>
       <c r="E193" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F193" s="41" t="s">
+      <c r="F193" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="194" spans="1:6" ht="34">
-      <c r="A194" s="39" t="str">
+      <c r="A194" s="2" t="str">
         <f>IF(ISNA(VLOOKUP(B194,AssociatedElements!B$2:B851,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
@@ -7878,18 +7868,18 @@
       <c r="C194" s="2" t="s">
         <v>903</v>
       </c>
-      <c r="D194" s="40" t="s">
+      <c r="D194" s="2" t="s">
         <v>904</v>
       </c>
       <c r="E194" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F194" s="41" t="s">
+      <c r="F194" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="195" spans="1:6" ht="34">
-      <c r="A195" s="39" t="str">
+      <c r="A195" s="2" t="str">
         <f>IF(ISNA(VLOOKUP(B195,AssociatedElements!B$2:B852,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
@@ -7899,18 +7889,18 @@
       <c r="C195" s="2" t="s">
         <v>906</v>
       </c>
-      <c r="D195" s="40" t="s">
+      <c r="D195" s="2" t="s">
         <v>907</v>
       </c>
       <c r="E195" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F195" s="41" t="s">
+      <c r="F195" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="196" spans="1:6" ht="34">
-      <c r="A196" s="39" t="str">
+      <c r="A196" s="2" t="str">
         <f>IF(ISNA(VLOOKUP(B196,AssociatedElements!B$2:B853,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
@@ -7920,18 +7910,18 @@
       <c r="C196" s="2" t="s">
         <v>909</v>
       </c>
-      <c r="D196" s="40" t="s">
+      <c r="D196" s="2" t="s">
         <v>910</v>
       </c>
       <c r="E196" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F196" s="41" t="s">
+      <c r="F196" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="197" spans="1:6" ht="34">
-      <c r="A197" s="39" t="str">
+      <c r="A197" s="2" t="str">
         <f>IF(ISNA(VLOOKUP(B197,AssociatedElements!B$2:B854,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
@@ -7941,18 +7931,18 @@
       <c r="C197" s="2" t="s">
         <v>912</v>
       </c>
-      <c r="D197" s="40" t="s">
+      <c r="D197" s="2" t="s">
         <v>913</v>
       </c>
       <c r="E197" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F197" s="41" t="s">
+      <c r="F197" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="198" spans="1:6" ht="34">
-      <c r="A198" s="39" t="str">
+      <c r="A198" s="2" t="str">
         <f>IF(ISNA(VLOOKUP(B198,AssociatedElements!B$2:B855,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
@@ -7962,18 +7952,18 @@
       <c r="C198" s="2" t="s">
         <v>915</v>
       </c>
-      <c r="D198" s="40" t="s">
+      <c r="D198" s="2" t="s">
         <v>916</v>
       </c>
       <c r="E198" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F198" s="41" t="s">
+      <c r="F198" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="199" spans="1:6" ht="34">
-      <c r="A199" s="39" t="str">
+      <c r="A199" s="2" t="str">
         <f>IF(ISNA(VLOOKUP(B199,AssociatedElements!B$2:B856,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
@@ -7983,13 +7973,13 @@
       <c r="C199" s="2" t="s">
         <v>918</v>
       </c>
-      <c r="D199" s="40" t="s">
+      <c r="D199" s="2" t="s">
         <v>919</v>
       </c>
       <c r="E199" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F199" s="41" t="s">
+      <c r="F199" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -12439,11 +12429,11 @@
       </c>
     </row>
     <row r="295" spans="1:4" ht="17">
-      <c r="A295" s="42" t="str">
+      <c r="A295" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B295,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B295" s="41" t="s">
+      <c r="B295" s="2" t="s">
         <v>892</v>
       </c>
       <c r="C295" s="4" t="s">
@@ -12454,11 +12444,11 @@
       </c>
     </row>
     <row r="296" spans="1:4" ht="17">
-      <c r="A296" s="42" t="str">
+      <c r="A296" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B296,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B296" s="41" t="s">
+      <c r="B296" s="2" t="s">
         <v>892</v>
       </c>
       <c r="C296" s="4" t="s">
@@ -12469,11 +12459,11 @@
       </c>
     </row>
     <row r="297" spans="1:4" ht="17">
-      <c r="A297" s="42" t="str">
+      <c r="A297" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B297,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B297" s="41" t="s">
+      <c r="B297" s="2" t="s">
         <v>894</v>
       </c>
       <c r="C297" s="4" t="s">
@@ -12484,11 +12474,11 @@
       </c>
     </row>
     <row r="298" spans="1:4" ht="17">
-      <c r="A298" s="42" t="str">
+      <c r="A298" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B298,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B298" s="41" t="s">
+      <c r="B298" s="2" t="s">
         <v>894</v>
       </c>
       <c r="C298" s="4" t="s">
@@ -12499,11 +12489,11 @@
       </c>
     </row>
     <row r="299" spans="1:4" ht="17">
-      <c r="A299" s="42" t="str">
+      <c r="A299" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B299,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B299" s="41" t="s">
+      <c r="B299" s="2" t="s">
         <v>896</v>
       </c>
       <c r="C299" s="4" t="s">
@@ -12514,11 +12504,11 @@
       </c>
     </row>
     <row r="300" spans="1:4" ht="17">
-      <c r="A300" s="42" t="str">
+      <c r="A300" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B300,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B300" s="41" t="s">
+      <c r="B300" s="2" t="s">
         <v>896</v>
       </c>
       <c r="C300" s="4" t="s">
@@ -12529,11 +12519,11 @@
       </c>
     </row>
     <row r="301" spans="1:4" ht="17">
-      <c r="A301" s="42" t="str">
+      <c r="A301" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B301,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B301" s="41" t="s">
+      <c r="B301" s="2" t="s">
         <v>899</v>
       </c>
       <c r="C301" s="4" t="s">
@@ -12544,11 +12534,11 @@
       </c>
     </row>
     <row r="302" spans="1:4" ht="17">
-      <c r="A302" s="42" t="str">
+      <c r="A302" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B302,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B302" s="41" t="s">
+      <c r="B302" s="2" t="s">
         <v>899</v>
       </c>
       <c r="C302" s="4" t="s">
@@ -12559,11 +12549,11 @@
       </c>
     </row>
     <row r="303" spans="1:4" ht="17">
-      <c r="A303" s="42" t="str">
+      <c r="A303" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B303,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B303" s="41" t="s">
+      <c r="B303" s="2" t="s">
         <v>902</v>
       </c>
       <c r="C303" s="4" t="s">
@@ -12574,11 +12564,11 @@
       </c>
     </row>
     <row r="304" spans="1:4" ht="17">
-      <c r="A304" s="42" t="str">
+      <c r="A304" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B304,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B304" s="41" t="s">
+      <c r="B304" s="2" t="s">
         <v>902</v>
       </c>
       <c r="C304" s="4" t="s">
@@ -12589,11 +12579,11 @@
       </c>
     </row>
     <row r="305" spans="1:4" ht="17">
-      <c r="A305" s="42" t="str">
+      <c r="A305" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B305,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B305" s="41" t="s">
+      <c r="B305" s="2" t="s">
         <v>905</v>
       </c>
       <c r="C305" s="4" t="s">
@@ -12604,11 +12594,11 @@
       </c>
     </row>
     <row r="306" spans="1:4" ht="17">
-      <c r="A306" s="42" t="str">
+      <c r="A306" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B306,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B306" s="41" t="s">
+      <c r="B306" s="2" t="s">
         <v>905</v>
       </c>
       <c r="C306" s="4" t="s">
@@ -12619,11 +12609,11 @@
       </c>
     </row>
     <row r="307" spans="1:4" ht="17">
-      <c r="A307" s="42" t="str">
+      <c r="A307" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B307,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B307" s="41" t="s">
+      <c r="B307" s="2" t="s">
         <v>908</v>
       </c>
       <c r="C307" s="4" t="s">
@@ -12634,11 +12624,11 @@
       </c>
     </row>
     <row r="308" spans="1:4" ht="17">
-      <c r="A308" s="42" t="str">
+      <c r="A308" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B308,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B308" s="41" t="s">
+      <c r="B308" s="2" t="s">
         <v>908</v>
       </c>
       <c r="C308" s="4" t="s">
@@ -12649,11 +12639,11 @@
       </c>
     </row>
     <row r="309" spans="1:4" ht="17">
-      <c r="A309" s="42" t="str">
+      <c r="A309" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B309,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B309" s="41" t="s">
+      <c r="B309" s="2" t="s">
         <v>911</v>
       </c>
       <c r="C309" s="4" t="s">
@@ -12664,11 +12654,11 @@
       </c>
     </row>
     <row r="310" spans="1:4" ht="17">
-      <c r="A310" s="42" t="str">
+      <c r="A310" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B310,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B310" s="41" t="s">
+      <c r="B310" s="2" t="s">
         <v>911</v>
       </c>
       <c r="C310" s="4" t="s">
@@ -12679,11 +12669,11 @@
       </c>
     </row>
     <row r="311" spans="1:4" ht="17">
-      <c r="A311" s="42" t="str">
+      <c r="A311" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B311,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B311" s="41" t="s">
+      <c r="B311" s="2" t="s">
         <v>914</v>
       </c>
       <c r="C311" s="4" t="s">
@@ -12694,11 +12684,11 @@
       </c>
     </row>
     <row r="312" spans="1:4" ht="17">
-      <c r="A312" s="42" t="str">
+      <c r="A312" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B312,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B312" s="41" t="s">
+      <c r="B312" s="2" t="s">
         <v>914</v>
       </c>
       <c r="C312" s="4" t="s">
@@ -12709,11 +12699,11 @@
       </c>
     </row>
     <row r="313" spans="1:4" ht="17">
-      <c r="A313" s="42" t="str">
+      <c r="A313" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B313,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B313" s="41" t="s">
+      <c r="B313" s="2" t="s">
         <v>917</v>
       </c>
       <c r="C313" s="4" t="s">
@@ -12724,11 +12714,11 @@
       </c>
     </row>
     <row r="314" spans="1:4" ht="17">
-      <c r="A314" s="42" t="str">
+      <c r="A314" t="str">
         <f>IF(ISNA(VLOOKUP([1]AssociatedElements!B314,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B314" s="41" t="s">
+      <c r="B314" s="2" t="s">
         <v>917</v>
       </c>
       <c r="C314" s="4" t="s">

</xml_diff>

<commit_message>
S30 - lateral load test dictionary, result property, and registry
New lateralLoadTestProcedure.xml (ASTM D3966/D3966M's eight named loading
procedures), new properties.xml#lateral_deflection (distinct from the
vertical-only #settlement), a widened equipmentClass.xml#load_test_reaction_frame
description covering the two-element push-apart lateral rig, and two new
registry entries (astm_d3966, nf_p94_151 - checked for an EN ISO 22477
counterpart and found the working-draft Part 3 was abandoned in 2007, never
published).
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/properties.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/properties.xlsx
@@ -1046,7 +1046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J211"/>
+  <dimension ref="A1:J212"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="7" customWidth="1" style="2" min="1" max="1"/>
@@ -7556,6 +7556,37 @@
         </is>
       </c>
     </row>
+    <row r="212">
+      <c r="A212">
+        <f>IF(ISNA(VLOOKUP(B212,AssociatedElements!B$2:B$1623,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>lateral_deflection</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Lateral Deflection</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Horizontal displacement of the load application point (or another stated gauge point) on a deep foundation element under a static lateral load test, measured against a stated datum. Distinct from properties.xml#settlement, which is explicitly vertical. A result of diggs:LateralLoadTest.</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -7571,7 +7602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D334"/>
+  <dimension ref="A1:D335"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="6.83203125" customWidth="1" min="1" max="1"/>
@@ -14556,6 +14587,27 @@
       <c r="D334" t="inlineStr">
         <is>
           <t>ancestor::diggs:measurement//diggs:procedure/diggs:ThermalIntegrityProfiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335">
+        <f>IF(ISNA(VLOOKUP(B335,Definitions!B$2:B$1623,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>lateral_deflection</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>//diggs:propertyClass</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:LateralLoadTest</t>
         </is>
       </c>
     </row>

</xml_diff>